<commit_message>
ajout KNN et RandomForest au tableau comparatif
</commit_message>
<xml_diff>
--- a/models/model_comparison.xlsx
+++ b/models/model_comparison.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,18 +28,9 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="009C0006"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00006100"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -51,23 +42,8 @@
         <fgColor rgb="00305496"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E7E6E6"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -75,42 +51,25 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="00BFBFBF"/>
-      </left>
-      <right style="thin">
-        <color rgb="00BFBFBF"/>
-      </right>
-      <top style="thin">
-        <color rgb="00BFBFBF"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00BFBFBF"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -478,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="54" customWidth="1" min="1" max="1"/>
@@ -550,27 +509,27 @@
           <t>non</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>max_iter=1000, solver=lbfgs (defaut)</t>
         </is>
       </c>
-      <c r="D2" s="4" t="n">
+      <c r="D2" s="5" t="n">
         <v>0.5998</v>
       </c>
-      <c r="E2" s="4" t="n">
+      <c r="E2" s="5" t="n">
         <v>0.38</v>
       </c>
-      <c r="F2" s="4" t="n">
+      <c r="F2" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="G2" s="4" t="n">
+      <c r="G2" s="5" t="n">
         <v>0.73</v>
       </c>
-      <c r="H2" s="4" t="n">
+      <c r="H2" s="5" t="n">
         <v>0.5600000000000001</v>
       </c>
-      <c r="I2" s="4" t="n">
+      <c r="I2" s="5" t="n">
         <v>0.21</v>
       </c>
     </row>
@@ -580,32 +539,32 @@
           <t>Regression logistique (balanced, OneVsRest)</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>balanced</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>max_iter=1000, solver=lbfgs (defaut)</t>
         </is>
       </c>
-      <c r="D3" s="4" t="n">
+      <c r="D3" s="5" t="n">
         <v>0.5192</v>
       </c>
-      <c r="E3" s="4" t="n">
+      <c r="E3" s="5" t="n">
         <v>0.44</v>
       </c>
-      <c r="F3" s="4" t="n">
+      <c r="F3" s="5" t="n">
         <v>0.17</v>
       </c>
-      <c r="G3" s="4" t="n">
+      <c r="G3" s="5" t="n">
         <v>0.63</v>
       </c>
-      <c r="H3" s="4" t="n">
+      <c r="H3" s="5" t="n">
         <v>0.55</v>
       </c>
-      <c r="I3" s="4" t="n">
+      <c r="I3" s="5" t="n">
         <v>0.38</v>
       </c>
     </row>
@@ -615,32 +574,32 @@
           <t>Regression logistique (GridSearch best, OneVsRest)</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>balanced</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>C=0.1, penalty=l2, solver=liblinear, max_iter=1000</t>
         </is>
       </c>
-      <c r="D4" s="4" t="n">
+      <c r="D4" s="5" t="n">
         <v>0.5173</v>
       </c>
-      <c r="E4" s="4" t="n">
+      <c r="E4" s="5" t="n">
         <v>0.43</v>
       </c>
-      <c r="F4" s="4" t="n">
+      <c r="F4" s="5" t="n">
         <v>0.17</v>
       </c>
-      <c r="G4" s="4" t="n">
+      <c r="G4" s="5" t="n">
         <v>0.63</v>
       </c>
-      <c r="H4" s="4" t="n">
+      <c r="H4" s="5" t="n">
         <v>0.55</v>
       </c>
-      <c r="I4" s="4" t="n">
+      <c r="I4" s="5" t="n">
         <v>0.38</v>
       </c>
     </row>
@@ -650,32 +609,32 @@
           <t>KNN (baseline)</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>non applicable (KNN)</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>n_neighbors=5, weights=uniform, metric=minkowski</t>
         </is>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="D5" s="5" t="n">
         <v>0.55</v>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="E5" s="5" t="n">
         <v>0.44</v>
       </c>
-      <c r="F5" s="4" t="n">
+      <c r="F5" s="5" t="n">
         <v>0.23</v>
       </c>
-      <c r="G5" s="4" t="n">
+      <c r="G5" s="5" t="n">
         <v>0.68</v>
       </c>
-      <c r="H5" s="4" t="n">
+      <c r="H5" s="5" t="n">
         <v>0.5</v>
       </c>
-      <c r="I5" s="4" t="n">
+      <c r="I5" s="5" t="n">
         <v>0.33</v>
       </c>
     </row>
@@ -685,32 +644,32 @@
           <t>KNN (GridSearch best)</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>non applicable (KNN)</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>n_neighbors=14, weights=uniform, metric=chebyshev</t>
         </is>
       </c>
-      <c r="D6" s="4" t="n">
+      <c r="D6" s="5" t="n">
         <v>0.6</v>
       </c>
-      <c r="E6" s="4" t="n">
+      <c r="E6" s="5" t="n">
         <v>0.46</v>
       </c>
-      <c r="F6" s="4" t="n">
+      <c r="F6" s="5" t="n">
         <v>0.18</v>
       </c>
-      <c r="G6" s="4" t="n">
+      <c r="G6" s="5" t="n">
         <v>0.73</v>
       </c>
-      <c r="H6" s="4" t="n">
+      <c r="H6" s="5" t="n">
         <v>0.54</v>
       </c>
-      <c r="I6" s="4" t="n">
+      <c r="I6" s="5" t="n">
         <v>0.39</v>
       </c>
     </row>
@@ -725,32 +684,102 @@
           <t>non</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>C=1, gamma=0.5, kernel=rbf</t>
         </is>
       </c>
-      <c r="D7" s="4" t="n">
-        <v>0.6209</v>
-      </c>
-      <c r="E7" s="4" t="n">
+      <c r="D7" s="5" t="n">
+        <v>0.6622</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="G7" s="5" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="H7" s="5" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="I7" s="5" t="n">
+        <v>0.91</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Random Forest (GridSearch best, balanced)</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>balanced</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>n_estimators=200, max_depth=20, max_features=sqrt, min_samples_leaf=4, min_samples_split=15</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>0.5744</v>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="G8" s="5" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H8" s="5" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="I8" s="5" t="n">
+        <v>0.46</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Random Forest (sans ponderation, validation)</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>n_estimators=200, max_depth=20, min_samples_leaf=4, min_samples_split=15 (sans GridSearch)</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>0.6102</v>
+      </c>
+      <c r="E9" s="5" t="n">
         <v>0.45</v>
       </c>
-      <c r="F7" s="4" t="n">
-        <v>0.09</v>
-      </c>
-      <c r="G7" s="4" t="n">
+      <c r="F9" s="5" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="G9" s="5" t="n">
         <v>0.74</v>
       </c>
-      <c r="H7" s="4" t="n">
+      <c r="H9" s="5" t="n">
         <v>0.5600000000000001</v>
       </c>
-      <c r="I7" s="4" t="n">
-        <v>0.41</v>
+      <c r="I9" s="5" t="n">
+        <v>0.39</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="D2:D7">
+  <conditionalFormatting sqref="D2:D9">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -762,7 +791,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E7">
+  <conditionalFormatting sqref="E2:E9">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -774,7 +803,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F2:F7">
+  <conditionalFormatting sqref="F2:F9">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -786,7 +815,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G7">
+  <conditionalFormatting sqref="G2:G9">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -798,7 +827,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H2:H7">
+  <conditionalFormatting sqref="H2:H9">
     <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -810,7 +839,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I2:I7">
+  <conditionalFormatting sqref="I2:I9">
     <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="num" val="0"/>

</xml_diff>